<commit_message>
feat: user can export PAR as PDF
</commit_message>
<xml_diff>
--- a/procurement_documents/PAR Template.xlsx
+++ b/procurement_documents/PAR Template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6B7624-F6F3-408F-A1DB-874BF7DE6BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F247355-4310-4FFF-8FB0-2955282AB1E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{58AB4997-63F7-4523-90D1-C9BD1C387E97}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{58AB4997-63F7-4523-90D1-C9BD1C387E97}"/>
   </bookViews>
   <sheets>
     <sheet name="PAR" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="40">
   <si>
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Fund Cluster :</t>
   </si>
   <si>
-    <t>Control No:</t>
-  </si>
-  <si>
     <t>P.O. No :</t>
   </si>
   <si>
@@ -111,9 +108,6 @@
     <t>Issued by:</t>
   </si>
   <si>
-    <t>Head ng supply</t>
-  </si>
-  <si>
     <t>Signature Over Printed Name</t>
   </si>
   <si>
@@ -123,7 +117,55 @@
     <t>Date</t>
   </si>
   <si>
-    <t>par_position</t>
+    <t>par_fund_cluster</t>
+  </si>
+  <si>
+    <t>par_po_no</t>
+  </si>
+  <si>
+    <t>PAR No:</t>
+  </si>
+  <si>
+    <t>par_no</t>
+  </si>
+  <si>
+    <t>par_code</t>
+  </si>
+  <si>
+    <t>par_received_by</t>
+  </si>
+  <si>
+    <t>par_received_by_pos</t>
+  </si>
+  <si>
+    <t>par_issued_by_pos</t>
+  </si>
+  <si>
+    <t>par_quantity</t>
+  </si>
+  <si>
+    <t>par_unit</t>
+  </si>
+  <si>
+    <t>par_items_descrip, + par_spec_description</t>
+  </si>
+  <si>
+    <t>par_property_no</t>
+  </si>
+  <si>
+    <t>par_date_acquired</t>
+  </si>
+  <si>
+    <t>par_amount</t>
+  </si>
+  <si>
+    <t>par_received_by_date</t>
+  </si>
+  <si>
+    <t>par_issued_by_date</t>
+  </si>
+  <si>
+    <t>par_issued_by</t>
   </si>
 </sst>
 </file>
@@ -611,40 +653,34 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -653,46 +689,52 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1153,122 +1195,122 @@
   <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" customWidth="1"/>
-    <col min="3" max="3" width="52.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" customWidth="1"/>
+    <col min="3" max="3" width="59.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="78"/>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
+      <c r="A1" s="57"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="80" t="s">
+      <c r="A2" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="74" t="s">
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="74" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
     </row>
     <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="74" t="s">
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="73"/>
-      <c r="D5" s="75" t="s">
+      <c r="B5" s="63"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="76" t="s">
+      <c r="A6" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="76"/>
-      <c r="C6" s="76"/>
-      <c r="D6" s="77"/>
-      <c r="E6" s="77"/>
-      <c r="F6" s="77"/>
+      <c r="B6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="70"/>
+      <c r="B7" s="68"/>
       <c r="C7" s="1"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="70"/>
+      <c r="B8" s="68"/>
       <c r="C8" s="5"/>
       <c r="D8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="83"/>
-      <c r="F8" s="84"/>
+        <v>11</v>
+      </c>
+      <c r="E8" s="69"/>
+      <c r="F8" s="70"/>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>17</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1545,87 +1587,87 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B44" s="72"/>
       <c r="C44" s="54"/>
       <c r="D44" s="53" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E44" s="55"/>
       <c r="F44" s="56"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="57"/>
-      <c r="B45" s="58"/>
-      <c r="C45" s="59"/>
-      <c r="D45" s="57"/>
-      <c r="E45" s="58"/>
-      <c r="F45" s="59"/>
+      <c r="A45" s="73"/>
+      <c r="B45" s="74"/>
+      <c r="C45" s="75"/>
+      <c r="D45" s="73"/>
+      <c r="E45" s="74"/>
+      <c r="F45" s="75"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="57"/>
-      <c r="B46" s="58"/>
-      <c r="C46" s="59"/>
-      <c r="D46" s="57"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="59"/>
+      <c r="A46" s="73"/>
+      <c r="B46" s="74"/>
+      <c r="C46" s="75"/>
+      <c r="D46" s="73"/>
+      <c r="E46" s="74"/>
+      <c r="F46" s="75"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="66"/>
-      <c r="B47" s="67"/>
-      <c r="C47" s="68"/>
-      <c r="D47" s="66"/>
-      <c r="E47" s="67"/>
-      <c r="F47" s="68"/>
+      <c r="A47" s="76"/>
+      <c r="B47" s="77"/>
+      <c r="C47" s="78"/>
+      <c r="D47" s="76"/>
+      <c r="E47" s="77"/>
+      <c r="F47" s="78"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="57" t="s">
+      <c r="A48" s="73" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="74"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="73"/>
+      <c r="E48" s="74"/>
+      <c r="F48" s="75"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="76"/>
+      <c r="B49" s="77"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="73"/>
+      <c r="E49" s="74"/>
+      <c r="F49" s="75"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="73" t="s">
+        <v>21</v>
+      </c>
+      <c r="B50" s="74"/>
+      <c r="C50" s="75"/>
+      <c r="D50" s="82"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="84"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="82"/>
+      <c r="B51" s="83"/>
+      <c r="C51" s="84"/>
+      <c r="D51" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="B48" s="58"/>
-      <c r="C48" s="59"/>
-      <c r="D48" s="57"/>
-      <c r="E48" s="58"/>
-      <c r="F48" s="59"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="66"/>
-      <c r="B49" s="67"/>
-      <c r="C49" s="68"/>
-      <c r="D49" s="57"/>
-      <c r="E49" s="58"/>
-      <c r="F49" s="59"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="57" t="s">
-        <v>23</v>
-      </c>
-      <c r="B50" s="58"/>
-      <c r="C50" s="59"/>
-      <c r="D50" s="60"/>
-      <c r="E50" s="61"/>
-      <c r="F50" s="62"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="60"/>
-      <c r="B51" s="61"/>
-      <c r="C51" s="62"/>
-      <c r="D51" s="57" t="s">
-        <v>24</v>
-      </c>
-      <c r="E51" s="58"/>
-      <c r="F51" s="59"/>
+      <c r="E51" s="74"/>
+      <c r="F51" s="75"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="63" t="s">
-        <v>24</v>
-      </c>
-      <c r="B52" s="64"/>
-      <c r="C52" s="65"/>
-      <c r="D52" s="63"/>
-      <c r="E52" s="64"/>
-      <c r="F52" s="65"/>
+      <c r="A52" s="79" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" s="80"/>
+      <c r="C52" s="81"/>
+      <c r="D52" s="79"/>
+      <c r="E52" s="80"/>
+      <c r="F52" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="32">
@@ -1670,6 +1712,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{028FE1CD-AA60-4A89-A65A-9651003B5219}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1682,122 +1725,142 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="78"/>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
+      <c r="A1" s="57"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="80" t="s">
+      <c r="A2" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="74" t="s">
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="74" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
     </row>
     <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="74" t="s">
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="73"/>
-      <c r="D5" s="75" t="s">
+      <c r="B5" s="63"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="76" t="s">
+      <c r="A6" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="76"/>
-      <c r="C6" s="76"/>
-      <c r="D6" s="77"/>
-      <c r="E6" s="77"/>
-      <c r="F6" s="77"/>
+      <c r="B6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="1"/>
+      <c r="B7" s="68"/>
+      <c r="C7" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="D7" s="2"/>
       <c r="E7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
+      <c r="B8" s="68"/>
+      <c r="C8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="70"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="83"/>
-      <c r="F8" s="84"/>
+      <c r="E8" s="69" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="70"/>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16"/>
+      <c r="A10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
@@ -2065,91 +2128,99 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B44" s="72"/>
       <c r="C44" s="54"/>
       <c r="D44" s="53" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E44" s="55"/>
       <c r="F44" s="56"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="57"/>
-      <c r="B45" s="58"/>
-      <c r="C45" s="59"/>
-      <c r="D45" s="57"/>
-      <c r="E45" s="58"/>
-      <c r="F45" s="59"/>
+      <c r="A45" s="73"/>
+      <c r="B45" s="74"/>
+      <c r="C45" s="75"/>
+      <c r="D45" s="73"/>
+      <c r="E45" s="74"/>
+      <c r="F45" s="75"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="57"/>
-      <c r="B46" s="58"/>
-      <c r="C46" s="59"/>
-      <c r="D46" s="57"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="59"/>
+      <c r="A46" s="73"/>
+      <c r="B46" s="74"/>
+      <c r="C46" s="75"/>
+      <c r="D46" s="73"/>
+      <c r="E46" s="74"/>
+      <c r="F46" s="75"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="66"/>
-      <c r="B47" s="67"/>
-      <c r="C47" s="68"/>
-      <c r="D47" s="66" t="s">
+      <c r="A47" s="76" t="s">
+        <v>28</v>
+      </c>
+      <c r="B47" s="77"/>
+      <c r="C47" s="78"/>
+      <c r="D47" s="76" t="s">
+        <v>39</v>
+      </c>
+      <c r="E47" s="77"/>
+      <c r="F47" s="78"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="73" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="74"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="73" t="s">
+        <v>30</v>
+      </c>
+      <c r="E48" s="74"/>
+      <c r="F48" s="75"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="76" t="s">
+        <v>29</v>
+      </c>
+      <c r="B49" s="77"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="73"/>
+      <c r="E49" s="74"/>
+      <c r="F49" s="75"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="E47" s="67"/>
-      <c r="F47" s="68"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="57" t="s">
+      <c r="B50" s="74"/>
+      <c r="C50" s="75"/>
+      <c r="D50" s="82" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" s="83"/>
+      <c r="F50" s="84"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="82" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" s="83"/>
+      <c r="C51" s="84"/>
+      <c r="D51" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="B48" s="58"/>
-      <c r="C48" s="59"/>
-      <c r="D48" s="57" t="s">
-        <v>25</v>
-      </c>
-      <c r="E48" s="58"/>
-      <c r="F48" s="59"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="66"/>
-      <c r="B49" s="67"/>
-      <c r="C49" s="68"/>
-      <c r="D49" s="57"/>
-      <c r="E49" s="58"/>
-      <c r="F49" s="59"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="57" t="s">
-        <v>23</v>
-      </c>
-      <c r="B50" s="58"/>
-      <c r="C50" s="59"/>
-      <c r="D50" s="60"/>
-      <c r="E50" s="61"/>
-      <c r="F50" s="62"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="60"/>
-      <c r="B51" s="61"/>
-      <c r="C51" s="62"/>
-      <c r="D51" s="57" t="s">
-        <v>24</v>
-      </c>
-      <c r="E51" s="58"/>
-      <c r="F51" s="59"/>
+      <c r="E51" s="74"/>
+      <c r="F51" s="75"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="63" t="s">
-        <v>24</v>
-      </c>
-      <c r="B52" s="64"/>
-      <c r="C52" s="65"/>
-      <c r="D52" s="63"/>
-      <c r="E52" s="64"/>
-      <c r="F52" s="65"/>
+      <c r="A52" s="79" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" s="80"/>
+      <c r="C52" s="81"/>
+      <c r="D52" s="79"/>
+      <c r="E52" s="80"/>
+      <c r="F52" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="32">

</xml_diff>

<commit_message>
feat: generate MR QR code for PAR
</commit_message>
<xml_diff>
--- a/procurement_documents/PAR Template.xlsx
+++ b/procurement_documents/PAR Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F247355-4310-4FFF-8FB0-2955282AB1E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{416665DD-4186-484E-B8E5-966F070AC95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{58AB4997-63F7-4523-90D1-C9BD1C387E97}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{58AB4997-63F7-4523-90D1-C9BD1C387E97}"/>
   </bookViews>
   <sheets>
     <sheet name="PAR" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="42">
   <si>
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
@@ -166,13 +166,20 @@
   </si>
   <si>
     <t>par_issued_by</t>
+  </si>
+  <si>
+    <t>Scan to receive item/s</t>
+  </si>
+  <si>
+    <t>Scan to
+receive item/s</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -303,6 +310,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -493,7 +508,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -653,6 +668,75 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -665,77 +749,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -752,154 +775,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>220318</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>81997</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="458857" cy="454004"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="C:\Users\arnel olivar\Desktop\logo tup.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{342E4049-D03B-464B-AAD0-64E164D251D3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="220318" y="81997"/>
-          <a:ext cx="458857" cy="454004"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>220318</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>81997</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="458857" cy="454004"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="C:\Users\arnel olivar\Desktop\logo tup.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE3DB9AD-3A5E-4C91-A90B-0E577772EE19}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="220318" y="81997"/>
-          <a:ext cx="458857" cy="454004"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1192,88 +1067,88 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A1ECFEB-B769-4E0A-9483-B15F55587700}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" customWidth="1"/>
-    <col min="3" max="3" width="59.5703125" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="62.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="57"/>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
+      <c r="A1" s="80"/>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="61" t="s">
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="61" t="s">
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
     </row>
     <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="61" t="s">
+      <c r="B4" s="75"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="63"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="64" t="s">
+      <c r="B5" s="75"/>
+      <c r="C5" s="75"/>
+      <c r="D5" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
+      <c r="B6" s="78"/>
+      <c r="C6" s="78"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="68"/>
+      <c r="B7" s="70"/>
       <c r="C7" s="1"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3" t="s">
@@ -1282,16 +1157,16 @@
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="67" t="s">
+      <c r="A8" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="68"/>
+      <c r="B8" s="70"/>
       <c r="C8" s="5"/>
       <c r="D8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="69"/>
-      <c r="F8" s="70"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="72"/>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
@@ -1586,10 +1461,10 @@
       <c r="F43" s="52"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="71" t="s">
+      <c r="A44" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="B44" s="72"/>
+      <c r="B44" s="74"/>
       <c r="C44" s="54"/>
       <c r="D44" s="53" t="s">
         <v>19</v>
@@ -1598,85 +1473,99 @@
       <c r="F44" s="56"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="73"/>
-      <c r="B45" s="74"/>
-      <c r="C45" s="75"/>
-      <c r="D45" s="73"/>
-      <c r="E45" s="74"/>
-      <c r="F45" s="75"/>
+      <c r="A45" s="63"/>
+      <c r="B45" s="64"/>
+      <c r="C45" s="65"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="64"/>
+      <c r="F45" s="65"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="73"/>
-      <c r="B46" s="74"/>
-      <c r="C46" s="75"/>
-      <c r="D46" s="73"/>
-      <c r="E46" s="74"/>
-      <c r="F46" s="75"/>
+      <c r="A46" s="63"/>
+      <c r="B46" s="64"/>
+      <c r="C46" s="65"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="64"/>
+      <c r="F46" s="65"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="76"/>
-      <c r="B47" s="77"/>
-      <c r="C47" s="78"/>
-      <c r="D47" s="76"/>
-      <c r="E47" s="77"/>
-      <c r="F47" s="78"/>
+      <c r="A47" s="60"/>
+      <c r="B47" s="61"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="61"/>
+      <c r="F47" s="62"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="73" t="s">
+      <c r="A48" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="74"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="73"/>
-      <c r="E48" s="74"/>
-      <c r="F48" s="75"/>
+      <c r="B48" s="64"/>
+      <c r="C48" s="65"/>
+      <c r="D48" s="63"/>
+      <c r="E48" s="64"/>
+      <c r="F48" s="65"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="76"/>
-      <c r="B49" s="77"/>
-      <c r="C49" s="78"/>
-      <c r="D49" s="73"/>
-      <c r="E49" s="74"/>
-      <c r="F49" s="75"/>
+      <c r="A49" s="60"/>
+      <c r="B49" s="61"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="64"/>
+      <c r="F49" s="65"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="73" t="s">
+      <c r="A50" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="74"/>
-      <c r="C50" s="75"/>
-      <c r="D50" s="82"/>
-      <c r="E50" s="83"/>
-      <c r="F50" s="84"/>
+      <c r="B50" s="64"/>
+      <c r="C50" s="65"/>
+      <c r="D50" s="66"/>
+      <c r="E50" s="67"/>
+      <c r="F50" s="68"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="82"/>
-      <c r="B51" s="83"/>
-      <c r="C51" s="84"/>
-      <c r="D51" s="73" t="s">
+      <c r="A51" s="66"/>
+      <c r="B51" s="67"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="E51" s="74"/>
-      <c r="F51" s="75"/>
+      <c r="E51" s="64"/>
+      <c r="F51" s="65"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="79" t="s">
+      <c r="A52" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="B52" s="80"/>
-      <c r="C52" s="81"/>
-      <c r="D52" s="79"/>
-      <c r="E52" s="80"/>
-      <c r="F52" s="81"/>
+      <c r="B52" s="58"/>
+      <c r="C52" s="59"/>
+      <c r="D52" s="57"/>
+      <c r="E52" s="58"/>
+      <c r="F52" s="59"/>
+    </row>
+    <row r="53" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="87"/>
+      <c r="B53" s="87"/>
+      <c r="C53" s="88" t="s">
+        <v>41</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
+  <mergeCells count="33">
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="D49:F49"/>
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="D46:F46"/>
     <mergeCell ref="A4:C4"/>
@@ -1691,29 +1580,22 @@
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="D45:F45"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{028FE1CD-AA60-4A89-A65A-9651003B5219}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -1725,76 +1607,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="57"/>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
+      <c r="A1" s="80"/>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="61" t="s">
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="61" t="s">
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
     </row>
     <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="61" t="s">
+      <c r="B4" s="75"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="63"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="64" t="s">
+      <c r="B5" s="75"/>
+      <c r="C5" s="75"/>
+      <c r="D5" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
+      <c r="B6" s="78"/>
+      <c r="C6" s="78"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="68"/>
+      <c r="B7" s="70"/>
       <c r="C7" s="1" t="s">
         <v>23</v>
       </c>
@@ -1807,20 +1689,20 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="67" t="s">
+      <c r="A8" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="68"/>
+      <c r="B8" s="70"/>
       <c r="C8" s="5" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="69" t="s">
+      <c r="E8" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="70"/>
+      <c r="F8" s="72"/>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
@@ -2127,10 +2009,10 @@
       <c r="F43" s="52"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="71" t="s">
+      <c r="A44" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="B44" s="72"/>
+      <c r="B44" s="74"/>
       <c r="C44" s="54"/>
       <c r="D44" s="53" t="s">
         <v>19</v>
@@ -2139,91 +2021,123 @@
       <c r="F44" s="56"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="73"/>
-      <c r="B45" s="74"/>
-      <c r="C45" s="75"/>
-      <c r="D45" s="73"/>
-      <c r="E45" s="74"/>
-      <c r="F45" s="75"/>
+      <c r="A45" s="63"/>
+      <c r="B45" s="64"/>
+      <c r="C45" s="65"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="64"/>
+      <c r="F45" s="65"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="73"/>
-      <c r="B46" s="74"/>
-      <c r="C46" s="75"/>
-      <c r="D46" s="73"/>
-      <c r="E46" s="74"/>
-      <c r="F46" s="75"/>
+      <c r="A46" s="63"/>
+      <c r="B46" s="64"/>
+      <c r="C46" s="65"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="64"/>
+      <c r="F46" s="65"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="76" t="s">
+      <c r="A47" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="B47" s="77"/>
-      <c r="C47" s="78"/>
-      <c r="D47" s="76" t="s">
+      <c r="B47" s="61"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="E47" s="77"/>
-      <c r="F47" s="78"/>
+      <c r="E47" s="61"/>
+      <c r="F47" s="62"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="73" t="s">
+      <c r="A48" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="74"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="73" t="s">
+      <c r="B48" s="64"/>
+      <c r="C48" s="65"/>
+      <c r="D48" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="E48" s="74"/>
-      <c r="F48" s="75"/>
+      <c r="E48" s="64"/>
+      <c r="F48" s="65"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="76" t="s">
+      <c r="A49" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="B49" s="77"/>
-      <c r="C49" s="78"/>
-      <c r="D49" s="73"/>
-      <c r="E49" s="74"/>
-      <c r="F49" s="75"/>
+      <c r="B49" s="61"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="64"/>
+      <c r="F49" s="65"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="73" t="s">
+      <c r="A50" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="74"/>
-      <c r="C50" s="75"/>
-      <c r="D50" s="82" t="s">
+      <c r="B50" s="64"/>
+      <c r="C50" s="65"/>
+      <c r="D50" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="E50" s="83"/>
-      <c r="F50" s="84"/>
+      <c r="E50" s="67"/>
+      <c r="F50" s="68"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="82" t="s">
+      <c r="A51" s="66" t="s">
         <v>37</v>
       </c>
-      <c r="B51" s="83"/>
-      <c r="C51" s="84"/>
-      <c r="D51" s="73" t="s">
+      <c r="B51" s="67"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="E51" s="74"/>
-      <c r="F51" s="75"/>
+      <c r="E51" s="64"/>
+      <c r="F51" s="65"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="79" t="s">
+      <c r="A52" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="B52" s="80"/>
-      <c r="C52" s="81"/>
-      <c r="D52" s="79"/>
-      <c r="E52" s="80"/>
-      <c r="F52" s="81"/>
+      <c r="B52" s="58"/>
+      <c r="C52" s="59"/>
+      <c r="D52" s="57"/>
+      <c r="E52" s="58"/>
+      <c r="F52" s="59"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="86"/>
+      <c r="B53" s="86"/>
+      <c r="C53" s="85" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="33">
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="D48:F48"/>
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="D52:F52"/>
     <mergeCell ref="A49:C49"/>
@@ -2232,33 +2146,8 @@
     <mergeCell ref="D50:F50"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="D51:F51"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: add tup logo in PAR pdf
</commit_message>
<xml_diff>
--- a/procurement_documents/PAR Template.xlsx
+++ b/procurement_documents/PAR Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{416665DD-4186-484E-B8E5-966F070AC95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA948215-456F-4776-86A6-EB97F242E814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{58AB4997-63F7-4523-90D1-C9BD1C387E97}"/>
   </bookViews>
@@ -45,8 +45,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
   <si>
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
@@ -173,13 +195,17 @@
   <si>
     <t>Scan to
 receive item/s</t>
+  </si>
+  <si>
+    <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES
+                               TAGUIG CITY</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,6 +344,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -508,7 +542,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -668,6 +702,31 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -686,22 +745,25 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -710,33 +772,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -752,13 +793,66 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,6 +895,70 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1079,76 +1237,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="80"/>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
+      <c r="A1" s="89" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="107" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="82" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="76" t="s">
+      <c r="A2" s="90"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="108"/>
+      <c r="D2" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="84" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="84"/>
-      <c r="C3" s="84"/>
-      <c r="D3" s="76" t="s">
+      <c r="A3" s="90"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="108"/>
+      <c r="D3" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
     </row>
     <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="75" t="s">
+      <c r="A4" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="76" t="s">
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="77" t="s">
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="77"/>
-      <c r="F5" s="77"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="74"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="78" t="s">
+      <c r="A6" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="78"/>
-      <c r="C6" s="78"/>
-      <c r="D6" s="79"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
+      <c r="B6" s="75"/>
+      <c r="C6" s="75"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="76"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="70"/>
+      <c r="B7" s="80"/>
       <c r="C7" s="1"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3" t="s">
@@ -1157,16 +1315,16 @@
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="79" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="70"/>
+      <c r="B8" s="80"/>
       <c r="C8" s="5"/>
       <c r="D8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="71"/>
-      <c r="F8" s="72"/>
+      <c r="E8" s="77"/>
+      <c r="F8" s="78"/>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
@@ -1192,279 +1350,279 @@
       <c r="A10" s="12"/>
       <c r="B10" s="12"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16"/>
+      <c r="D10" s="94"/>
+      <c r="E10" s="98"/>
+      <c r="F10" s="102"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
+      <c r="B11" s="8"/>
       <c r="C11" s="17"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="16"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="98"/>
+      <c r="F11" s="102"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="20"/>
       <c r="D12" s="21"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="23"/>
+      <c r="E12" s="99"/>
+      <c r="F12" s="103"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="19"/>
-      <c r="B13" s="19"/>
+      <c r="B13" s="12"/>
       <c r="C13" s="24"/>
       <c r="D13" s="25"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="26"/>
+      <c r="E13" s="98"/>
+      <c r="F13" s="104"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
+      <c r="B14" s="12"/>
       <c r="C14" s="27"/>
       <c r="D14" s="28"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="23"/>
+      <c r="E14" s="99"/>
+      <c r="F14" s="103"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="29"/>
-      <c r="B15" s="29"/>
+      <c r="B15" s="93"/>
       <c r="C15" s="30"/>
       <c r="D15" s="21"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="26"/>
+      <c r="E15" s="98"/>
+      <c r="F15" s="104"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="29"/>
-      <c r="B16" s="29"/>
+      <c r="B16" s="93"/>
       <c r="C16" s="31"/>
       <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+      <c r="E16" s="100"/>
+      <c r="F16" s="103"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="93"/>
       <c r="C17" s="30"/>
       <c r="D17" s="34"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="23"/>
+      <c r="E17" s="100"/>
+      <c r="F17" s="103"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
+      <c r="B18" s="93"/>
       <c r="C18" s="24"/>
       <c r="D18" s="35"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="26"/>
+      <c r="E18" s="100"/>
+      <c r="F18" s="104"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="29"/>
-      <c r="B19" s="29"/>
+      <c r="B19" s="93"/>
       <c r="C19" s="30"/>
       <c r="D19" s="21"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="26"/>
+      <c r="E19" s="98"/>
+      <c r="F19" s="104"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="29"/>
-      <c r="B20" s="29"/>
+      <c r="B20" s="93"/>
       <c r="C20" s="13"/>
       <c r="D20" s="21"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="26"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="104"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
+      <c r="B21" s="93"/>
       <c r="C21" s="24"/>
       <c r="D21" s="25"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="26"/>
+      <c r="E21" s="100"/>
+      <c r="F21" s="104"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="19"/>
-      <c r="B22" s="19"/>
+      <c r="B22" s="12"/>
       <c r="C22" s="31"/>
       <c r="D22" s="36"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="23"/>
+      <c r="E22" s="99"/>
+      <c r="F22" s="103"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="19"/>
-      <c r="B23" s="19"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="37"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="23"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="100"/>
+      <c r="F23" s="103"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="19"/>
-      <c r="B24" s="19"/>
+      <c r="B24" s="12"/>
       <c r="C24" s="39"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="23"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="100"/>
+      <c r="F24" s="103"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="19"/>
-      <c r="B25" s="19"/>
+      <c r="B25" s="12"/>
       <c r="C25" s="13"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="26"/>
+      <c r="D25" s="95"/>
+      <c r="E25" s="98"/>
+      <c r="F25" s="104"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
+      <c r="B26" s="12"/>
       <c r="C26" s="41"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="23"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="100"/>
+      <c r="F26" s="103"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="19"/>
-      <c r="B27" s="19"/>
+      <c r="B27" s="12"/>
       <c r="C27" s="30"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="23"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="100"/>
+      <c r="F27" s="103"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="19"/>
-      <c r="B28" s="19"/>
+      <c r="B28" s="12"/>
       <c r="C28" s="42"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="23"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="100"/>
+      <c r="F28" s="103"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="19"/>
-      <c r="B29" s="19"/>
+      <c r="B29" s="12"/>
       <c r="C29" s="27"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="23"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="100"/>
+      <c r="F29" s="103"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="19"/>
-      <c r="B30" s="19"/>
+      <c r="B30" s="12"/>
       <c r="C30" s="43"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="23"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="100"/>
+      <c r="F30" s="103"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
+      <c r="B31" s="12"/>
       <c r="C31" s="44"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="23"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="100"/>
+      <c r="F31" s="103"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="19"/>
-      <c r="B32" s="19"/>
+      <c r="B32" s="12"/>
       <c r="C32" s="45"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="23"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="100"/>
+      <c r="F32" s="103"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="19"/>
-      <c r="B33" s="19"/>
+      <c r="B33" s="12"/>
       <c r="C33" s="44"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="23"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="100"/>
+      <c r="F33" s="103"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="19"/>
-      <c r="B34" s="19"/>
+      <c r="B34" s="12"/>
       <c r="C34" s="44"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="23"/>
+      <c r="D34" s="97"/>
+      <c r="E34" s="100"/>
+      <c r="F34" s="103"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="19"/>
-      <c r="B35" s="19"/>
+      <c r="B35" s="12"/>
       <c r="C35" s="39"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="23"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="100"/>
+      <c r="F35" s="103"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="19"/>
-      <c r="B36" s="19"/>
+      <c r="B36" s="12"/>
       <c r="C36" s="41"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="23"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="100"/>
+      <c r="F36" s="103"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="19"/>
-      <c r="B37" s="19"/>
+      <c r="B37" s="12"/>
       <c r="C37" s="41"/>
-      <c r="D37" s="38"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="23"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="100"/>
+      <c r="F37" s="103"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="19"/>
-      <c r="B38" s="19"/>
+      <c r="B38" s="12"/>
       <c r="C38" s="41"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="23"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="100"/>
+      <c r="F38" s="103"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="19"/>
-      <c r="B39" s="19"/>
+      <c r="B39" s="12"/>
       <c r="C39" s="39"/>
-      <c r="D39" s="38"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="23"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="100"/>
+      <c r="F39" s="103"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="19"/>
-      <c r="B40" s="19"/>
+      <c r="B40" s="12"/>
       <c r="C40" s="47"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="49"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="105"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="19"/>
-      <c r="B41" s="19"/>
+      <c r="B41" s="12"/>
       <c r="C41" s="39"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="33"/>
-      <c r="F41" s="49"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="100"/>
+      <c r="F41" s="105"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="19"/>
-      <c r="B42" s="19"/>
+      <c r="B42" s="12"/>
       <c r="C42" s="47"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="49"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="100"/>
+      <c r="F42" s="105"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="19"/>
-      <c r="B43" s="19"/>
+      <c r="B43" s="12"/>
       <c r="C43" s="47"/>
-      <c r="D43" s="50"/>
-      <c r="E43" s="51"/>
-      <c r="F43" s="52"/>
+      <c r="D43" s="96"/>
+      <c r="E43" s="101"/>
+      <c r="F43" s="106"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="73" t="s">
+      <c r="A44" s="81" t="s">
         <v>18</v>
       </c>
-      <c r="B44" s="74"/>
+      <c r="B44" s="82"/>
       <c r="C44" s="54"/>
       <c r="D44" s="53" t="s">
         <v>19</v>
@@ -1473,99 +1631,91 @@
       <c r="F44" s="56"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="63"/>
-      <c r="B45" s="64"/>
-      <c r="C45" s="65"/>
-      <c r="D45" s="63"/>
-      <c r="E45" s="64"/>
-      <c r="F45" s="65"/>
+      <c r="A45" s="60"/>
+      <c r="B45" s="61"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="60"/>
+      <c r="E45" s="61"/>
+      <c r="F45" s="62"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="63"/>
-      <c r="B46" s="64"/>
-      <c r="C46" s="65"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="64"/>
-      <c r="F46" s="65"/>
+      <c r="A46" s="60"/>
+      <c r="B46" s="61"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="60"/>
+      <c r="E46" s="61"/>
+      <c r="F46" s="62"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="60"/>
-      <c r="B47" s="61"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="60"/>
-      <c r="E47" s="61"/>
-      <c r="F47" s="62"/>
+      <c r="A47" s="69"/>
+      <c r="B47" s="70"/>
+      <c r="C47" s="71"/>
+      <c r="D47" s="69"/>
+      <c r="E47" s="70"/>
+      <c r="F47" s="71"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="63" t="s">
+      <c r="A48" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="64"/>
-      <c r="C48" s="65"/>
-      <c r="D48" s="63"/>
-      <c r="E48" s="64"/>
-      <c r="F48" s="65"/>
+      <c r="B48" s="61"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="60"/>
+      <c r="E48" s="61"/>
+      <c r="F48" s="62"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="60"/>
-      <c r="B49" s="61"/>
-      <c r="C49" s="62"/>
-      <c r="D49" s="63"/>
-      <c r="E49" s="64"/>
-      <c r="F49" s="65"/>
+      <c r="A49" s="69"/>
+      <c r="B49" s="70"/>
+      <c r="C49" s="71"/>
+      <c r="D49" s="60"/>
+      <c r="E49" s="61"/>
+      <c r="F49" s="62"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="63" t="s">
+      <c r="A50" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="64"/>
-      <c r="C50" s="65"/>
-      <c r="D50" s="66"/>
-      <c r="E50" s="67"/>
-      <c r="F50" s="68"/>
+      <c r="B50" s="61"/>
+      <c r="C50" s="62"/>
+      <c r="D50" s="63"/>
+      <c r="E50" s="64"/>
+      <c r="F50" s="65"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="66"/>
-      <c r="B51" s="67"/>
-      <c r="C51" s="68"/>
-      <c r="D51" s="63" t="s">
+      <c r="A51" s="63"/>
+      <c r="B51" s="64"/>
+      <c r="C51" s="65"/>
+      <c r="D51" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="E51" s="64"/>
-      <c r="F51" s="65"/>
+      <c r="E51" s="61"/>
+      <c r="F51" s="62"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="57" t="s">
+      <c r="A52" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="B52" s="58"/>
-      <c r="C52" s="59"/>
-      <c r="D52" s="57"/>
-      <c r="E52" s="58"/>
-      <c r="F52" s="59"/>
+      <c r="B52" s="67"/>
+      <c r="C52" s="68"/>
+      <c r="D52" s="66"/>
+      <c r="E52" s="67"/>
+      <c r="F52" s="68"/>
     </row>
     <row r="53" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="87"/>
-      <c r="B53" s="87"/>
-      <c r="C53" s="88" t="s">
+      <c r="A53" s="59"/>
+      <c r="B53" s="59"/>
+      <c r="C53" s="58" t="s">
         <v>41</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="D49:F49"/>
+  <mergeCells count="32">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="A1:B3"/>
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="D46:F46"/>
     <mergeCell ref="A4:C4"/>
@@ -1580,12 +1730,19 @@
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="D45:F45"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:F52"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1607,76 +1764,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="80"/>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
+      <c r="A1" s="83"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="76" t="s">
+      <c r="B2" s="86"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="84"/>
-      <c r="C3" s="84"/>
-      <c r="D3" s="76" t="s">
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
     </row>
     <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="75" t="s">
+      <c r="A4" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="76" t="s">
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="77" t="s">
+      <c r="B5" s="72"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="77"/>
-      <c r="F5" s="77"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="74"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="78" t="s">
+      <c r="A6" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="78"/>
-      <c r="C6" s="78"/>
-      <c r="D6" s="79"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
+      <c r="B6" s="75"/>
+      <c r="C6" s="75"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="76"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="70"/>
+      <c r="B7" s="80"/>
       <c r="C7" s="1" t="s">
         <v>23</v>
       </c>
@@ -1689,20 +1846,20 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="79" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="70"/>
+      <c r="B8" s="80"/>
       <c r="C8" s="5" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="71" t="s">
+      <c r="E8" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="72"/>
+      <c r="F8" s="78"/>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
@@ -2009,10 +2166,10 @@
       <c r="F43" s="52"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="73" t="s">
+      <c r="A44" s="81" t="s">
         <v>18</v>
       </c>
-      <c r="B44" s="74"/>
+      <c r="B44" s="82"/>
       <c r="C44" s="54"/>
       <c r="D44" s="53" t="s">
         <v>19</v>
@@ -2021,98 +2178,115 @@
       <c r="F44" s="56"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="63"/>
-      <c r="B45" s="64"/>
-      <c r="C45" s="65"/>
-      <c r="D45" s="63"/>
-      <c r="E45" s="64"/>
-      <c r="F45" s="65"/>
+      <c r="A45" s="60"/>
+      <c r="B45" s="61"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="60"/>
+      <c r="E45" s="61"/>
+      <c r="F45" s="62"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="63"/>
-      <c r="B46" s="64"/>
-      <c r="C46" s="65"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="64"/>
-      <c r="F46" s="65"/>
+      <c r="A46" s="60"/>
+      <c r="B46" s="61"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="60"/>
+      <c r="E46" s="61"/>
+      <c r="F46" s="62"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="60" t="s">
+      <c r="A47" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="B47" s="61"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="60" t="s">
+      <c r="B47" s="70"/>
+      <c r="C47" s="71"/>
+      <c r="D47" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="E47" s="61"/>
-      <c r="F47" s="62"/>
+      <c r="E47" s="70"/>
+      <c r="F47" s="71"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="63" t="s">
+      <c r="A48" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="64"/>
-      <c r="C48" s="65"/>
-      <c r="D48" s="63" t="s">
+      <c r="B48" s="61"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="E48" s="64"/>
-      <c r="F48" s="65"/>
+      <c r="E48" s="61"/>
+      <c r="F48" s="62"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="60" t="s">
+      <c r="A49" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="B49" s="61"/>
-      <c r="C49" s="62"/>
-      <c r="D49" s="63"/>
-      <c r="E49" s="64"/>
-      <c r="F49" s="65"/>
+      <c r="B49" s="70"/>
+      <c r="C49" s="71"/>
+      <c r="D49" s="60"/>
+      <c r="E49" s="61"/>
+      <c r="F49" s="62"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="63" t="s">
+      <c r="A50" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="64"/>
-      <c r="C50" s="65"/>
-      <c r="D50" s="66" t="s">
+      <c r="B50" s="61"/>
+      <c r="C50" s="62"/>
+      <c r="D50" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="E50" s="67"/>
-      <c r="F50" s="68"/>
+      <c r="E50" s="64"/>
+      <c r="F50" s="65"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="66" t="s">
+      <c r="A51" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="B51" s="67"/>
-      <c r="C51" s="68"/>
-      <c r="D51" s="63" t="s">
+      <c r="B51" s="64"/>
+      <c r="C51" s="65"/>
+      <c r="D51" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="E51" s="64"/>
-      <c r="F51" s="65"/>
+      <c r="E51" s="61"/>
+      <c r="F51" s="62"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="57" t="s">
+      <c r="A52" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="B52" s="58"/>
-      <c r="C52" s="59"/>
-      <c r="D52" s="57"/>
-      <c r="E52" s="58"/>
-      <c r="F52" s="59"/>
+      <c r="B52" s="67"/>
+      <c r="C52" s="68"/>
+      <c r="D52" s="66"/>
+      <c r="E52" s="67"/>
+      <c r="F52" s="68"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="86"/>
-      <c r="B53" s="86"/>
-      <c r="C53" s="85" t="s">
+      <c r="A53" s="88"/>
+      <c r="B53" s="88"/>
+      <c r="C53" s="57" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="D46:F46"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:F1"/>
@@ -2129,23 +2303,6 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:F51"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>